<commit_message>
feat: Proyecto Grande Solo - Sistema Ventas Empresarial completo con KPIs, Dashboard, Macro
</commit_message>
<xml_diff>
--- a/Formulas-Fecha-2026.xlsx
+++ b/Formulas-Fecha-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{E0D0F2AA-42ED-4E8E-A4F0-CC8BE3E457C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A29CBCF8-A39C-4BDF-91E7-AF7E6B0E366A}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{E0D0F2AA-42ED-4E8E-A4F0-CC8BE3E457C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2D520A9-DC3F-430E-AF76-E8F150647AE5}"/>
   <bookViews>
-    <workbookView xWindow="84" yWindow="0" windowWidth="12528" windowHeight="12240" xr2:uid="{3D26376A-7878-46AD-A1F1-4A341476EC69}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3D26376A-7878-46AD-A1F1-4A341476EC69}"/>
   </bookViews>
   <sheets>
     <sheet name="Fechas" sheetId="1" r:id="rId1"/>
@@ -125,7 +125,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -183,9 +183,6 @@
   </cellStyleXfs>
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -193,65 +190,46 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="15">
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF0070C0"/>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -311,7 +289,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="169" formatCode="dd/mm/yyyy;@"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -426,7 +404,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="169" formatCode="dd/mm/yyyy;@"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
     </dxf>
     <dxf>
       <font>
@@ -445,7 +423,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="169" formatCode="dd/mm/yyyy;@"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
     </dxf>
     <dxf>
       <font>
@@ -466,23 +444,38 @@
       </font>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
       <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF0070C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -500,7 +493,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D6A002B-9B34-4C55-AA5B-A5B5F478067B}" name="Empleados" displayName="Empleados" ref="A3:K13" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D6A002B-9B34-4C55-AA5B-A5B5F478067B}" name="Empleados" displayName="Empleados" ref="A3:K13" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
   <autoFilter ref="A3:K13" xr:uid="{8D6A002B-9B34-4C55-AA5B-A5B5F478067B}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{449DFCD7-B8B3-4312-9E05-49534A821891}" name="Empleado" dataDxfId="12"/>
@@ -834,642 +827,662 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" style="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.33203125" style="13" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.77734375" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.33203125" style="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.77734375" style="11" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="I3" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
         <v>45292</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <v>46174</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="10">
         <f t="shared" ref="E4:E13" si="0">DATEDIF(B4,C4,"Y")</f>
         <v>2</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <f t="shared" ref="F4:F13" si="1">DATEDIF(B4,C4, "M")</f>
         <v>29</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <f t="shared" ref="G4:G13" si="2">DATEDIF(B4,C4, "D")</f>
         <v>882</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="2">
         <f t="shared" ref="H4:H13" si="3">NETWORKDAYS(B4,C4)</f>
         <v>631</v>
       </c>
-      <c r="I4" s="15">
+      <c r="I4" s="14">
         <f>EDATE(C4,6)</f>
         <v>46357</v>
       </c>
-      <c r="J4" s="11" t="str">
+      <c r="J4" s="10" t="str">
         <f t="shared" ref="J4:J13" si="4">CHOOSE(WEEKDAY(B4,2), "Lunes", "Martes", "Miercoles", "Jueves", "Viernes", "Sabado", "Domingo")</f>
         <v>Lunes</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="3">
         <f t="shared" ref="K4:K13" ca="1" si="5">TODAY()</f>
-        <v>46198</v>
-      </c>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <v>45000</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <v>46096</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="10">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="2">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="2">
         <f t="shared" si="2"/>
         <v>1096</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="2">
         <f t="shared" si="3"/>
         <v>783</v>
       </c>
-      <c r="I5" s="15">
-        <f t="shared" ref="I4:I13" si="6">EDATE(C5,6)</f>
+      <c r="I5" s="14">
+        <f t="shared" ref="I5:I13" si="6">EDATE(C5,6)</f>
         <v>46280</v>
       </c>
-      <c r="J5" s="11" t="str">
+      <c r="J5" s="10" t="str">
         <f t="shared" si="4"/>
         <v>Miercoles</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="3">
         <f t="shared" ca="1" si="5"/>
-        <v>46198</v>
-      </c>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <v>44722</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="7">
         <v>46032</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="10">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="2">
         <f t="shared" si="1"/>
         <v>43</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="2">
         <f t="shared" si="2"/>
         <v>1310</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="2">
         <f t="shared" si="3"/>
         <v>936</v>
       </c>
-      <c r="I6" s="15">
+      <c r="I6" s="14">
         <f t="shared" si="6"/>
         <v>46213</v>
       </c>
-      <c r="J6" s="11" t="str">
+      <c r="J6" s="10" t="str">
         <f t="shared" si="4"/>
         <v>Viernes</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="3">
         <f t="shared" ca="1" si="5"/>
-        <v>46198</v>
-      </c>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="7">
         <v>44459</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="7">
         <v>45920</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="10">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="2">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="2">
         <f t="shared" si="2"/>
         <v>1461</v>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="2">
         <f t="shared" si="3"/>
         <v>1045</v>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="14">
         <f t="shared" si="6"/>
         <v>46101</v>
       </c>
-      <c r="J7" s="11" t="str">
+      <c r="J7" s="10" t="str">
         <f t="shared" si="4"/>
         <v>Lunes</v>
       </c>
-      <c r="K7" s="4">
+      <c r="K7" s="3">
         <f t="shared" ca="1" si="5"/>
-        <v>46198</v>
-      </c>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="7">
         <v>44170</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="7">
         <v>46178</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="10">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <f t="shared" si="1"/>
         <v>66</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="2">
         <f t="shared" si="2"/>
         <v>2008</v>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="2">
         <f t="shared" si="3"/>
         <v>1435</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="14">
         <f t="shared" si="6"/>
         <v>46361</v>
       </c>
-      <c r="J8" s="11" t="str">
+      <c r="J8" s="10" t="str">
         <f t="shared" si="4"/>
         <v>Sabado</v>
       </c>
-      <c r="K8" s="4">
+      <c r="K8" s="3">
         <f t="shared" ca="1" si="5"/>
-        <v>46198</v>
-      </c>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="7">
         <v>45034</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="7">
         <v>46130</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="10">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="2">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="2">
         <f t="shared" si="2"/>
         <v>1096</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="2">
         <f t="shared" si="3"/>
         <v>784</v>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="14">
         <f t="shared" si="6"/>
         <v>46313</v>
       </c>
-      <c r="J9" s="11" t="str">
+      <c r="J9" s="10" t="str">
         <f t="shared" si="4"/>
         <v>Martes</v>
       </c>
-      <c r="K9" s="4">
+      <c r="K9" s="3">
         <f t="shared" ca="1" si="5"/>
-        <v>46198</v>
-      </c>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="7">
         <v>43668</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="7">
         <v>45860</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="10">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="2">
         <f t="shared" si="2"/>
         <v>2192</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="2">
         <f t="shared" si="3"/>
         <v>1567</v>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="14">
         <f t="shared" si="6"/>
         <v>46044</v>
       </c>
-      <c r="J10" s="11" t="str">
+      <c r="J10" s="10" t="str">
         <f t="shared" si="4"/>
         <v>Lunes</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="3">
         <f t="shared" ca="1" si="5"/>
-        <v>46198</v>
-      </c>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="7">
         <v>45626</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="7">
         <v>46172</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="10">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="2">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="2">
         <f t="shared" si="2"/>
         <v>546</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="2">
         <f t="shared" si="3"/>
         <v>390</v>
       </c>
-      <c r="I11" s="15">
+      <c r="I11" s="14">
         <f t="shared" si="6"/>
         <v>46356</v>
       </c>
-      <c r="J11" s="11" t="str">
+      <c r="J11" s="10" t="str">
         <f t="shared" si="4"/>
         <v>Sabado</v>
       </c>
-      <c r="K11" s="4">
+      <c r="K11" s="3">
         <f t="shared" ca="1" si="5"/>
-        <v>46198</v>
-      </c>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="7">
         <v>44606</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="7">
         <v>46067</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="10">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="2">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="2">
         <f t="shared" si="2"/>
         <v>1461</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="2">
         <f t="shared" si="3"/>
         <v>1045</v>
       </c>
-      <c r="I12" s="15">
+      <c r="I12" s="14">
         <f t="shared" si="6"/>
         <v>46248</v>
       </c>
-      <c r="J12" s="11" t="str">
+      <c r="J12" s="10" t="str">
         <f t="shared" si="4"/>
         <v>Lunes</v>
       </c>
-      <c r="K12" s="4">
+      <c r="K12" s="3">
         <f t="shared" ca="1" si="5"/>
-        <v>46198</v>
-      </c>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="7">
         <v>45146</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="7">
         <v>46242</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="10">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="2">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="2">
         <f t="shared" si="2"/>
         <v>1096</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="2">
         <f t="shared" si="3"/>
         <v>784</v>
       </c>
-      <c r="I13" s="15">
+      <c r="I13" s="14">
         <f t="shared" si="6"/>
         <v>46426</v>
       </c>
-      <c r="J13" s="11" t="str">
+      <c r="J13" s="10" t="str">
         <f t="shared" si="4"/>
         <v>Martes</v>
       </c>
-      <c r="K13" s="4">
+      <c r="K13" s="3">
         <f t="shared" ca="1" si="5"/>
-        <v>46198</v>
-      </c>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
+        <v>46199</v>
+      </c>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="3"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
+      <c r="A14" s="2"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="3"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="11">
+      <c r="A16" s="2"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="10">
         <f>DATEDIF(B4,C4, "Y")</f>
         <v>2</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="2">
         <f>DATEDIF(B4,C4, "M")</f>
         <v>29</v>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" s="2">
         <f>DATEDIF(B4,C4, "D")</f>
         <v>882</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="2">
         <f>NETWORKDAYS(B4,C4)</f>
         <v>631</v>
       </c>
-      <c r="I16" s="15">
+      <c r="I16" s="14">
         <f>EDATE(C4, -3)</f>
         <v>46082</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="10">
         <f>WEEKDAY(B4,2)</f>
         <v>1</v>
       </c>
-      <c r="K16" s="4">
+      <c r="K16" s="3">
         <f ca="1">TODAY()</f>
-        <v>46198</v>
-      </c>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="3"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="F19" s="3"/>
-      <c r="H19" s="2"/>
+        <v>46199</v>
+      </c>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="2"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="10">
+        <f>DATEDIF(B4,C4, "Y")</f>
+        <v>2</v>
+      </c>
+      <c r="F17" s="2">
+        <f>DATEDIF(B4,C4, "M")</f>
+        <v>29</v>
+      </c>
+      <c r="G17" s="2">
+        <f>DATEDIF(B4,C4, "D")</f>
+        <v>882</v>
+      </c>
+      <c r="H17" s="2">
+        <f>NETWORKDAYS(B4,C4)</f>
+        <v>631</v>
+      </c>
+      <c r="I17" s="12">
+        <f>EDATE(C4,6)</f>
+        <v>46357</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="K18" s="1">
+        <f ca="1">TODAY()</f>
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="F19" s="2"/>
+      <c r="H19" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <conditionalFormatting sqref="I4:I13">
-    <cfRule type="expression" dxfId="15" priority="2">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>I4&gt;=TODAY()</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>I4&lt;TODAY()</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="1">
-      <formula>I4&gt;=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>